<commit_message>
chore: lock the profitability tracker sheets
All sheets and the workbook structure are password-protected so visitors can read the formulas but not change them. Values unchanged (total net revenue 2,274.42, 5 flagged orders).
</commit_message>
<xml_diff>
--- a/files/11 Profitability Tracker - Luna and Lace.xlsx
+++ b/files/11 Profitability Tracker - Luna and Lace.xlsx
@@ -3,6 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="5GfkPf7MadITjoX/dT7OWSs/lUicUZUmNIjDmC/3RtJpEwq8E/M6g8HVkszI24iXijsmzvOc0G8KgKjJbrEXsg==" workbookSaltValue="TkIO+Dm7kRWg8VmEvM0t4g==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView/>
   </bookViews>
@@ -458,7 +459,7 @@
     <numFmt numFmtId="179" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="180" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -514,13 +515,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF0F766E"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1000,28 +994,31 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1030,118 +1027,115 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1619,6 +1613,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="DJsQhE2zLG9z86JkmTxm6hjwunRm5Vglommu/yVMXLb/ABOSYeiHp8xw0FHwF2iEKzjmVi1PTICRgKtcphHhkg==" saltValue="eNuxsOqetoayTBjjujYUow==" spinCount="100000" sheet="1" objects="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -1680,6 +1675,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="LBV6rgXMgQ1IZJzLer2fmlQrzO4Ek0UJuy01Ldp3cSfJDCTMa00IB8qCQIECTczjJLtjMnaFh40QSdouMCsa9w==" saltValue="PeTjEnYTT2ROamoWWwXGDQ==" spinCount="100000" sheet="1" objects="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -1860,6 +1856,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="nzwxXeqEEuBaDZ7pHSVUYZbmsh2hMvPQxQ2Tw7cf8D6hXm6dNZ8U+hCJH5nNuMRDdyK6otvwIypxlC7MLGR2JQ==" saltValue="BvqB5ssg3A1/hDuaHCCujg==" spinCount="100000" sheet="1" objects="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -5229,6 +5226,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="k7Ppz+w7Nu07jcLBVbOH9PKM7DCHnNM4oASNctLBIptRmEqeBMvyjc3C0nc9wJOK5W0Bxv5QX23IhTCx0ll4UQ==" saltValue="5wQwYYf1w6qf7r7xv7FgLA==" spinCount="100000" sheet="1" objects="1"/>
   <conditionalFormatting sqref="A2:S50">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$S2&lt;&gt;""</formula>
@@ -5878,6 +5876,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="BGN8XGhjm3PoGAByDdfbBUWbN8HZTYqR4z8Kcz1x4aJPLawdluBnrWgtvSNXZ7BOTrfpxMRU0Q5pSAHQ50DfSw==" saltValue="XSZBIdu9///oEUyyld1W4w==" spinCount="100000" sheet="1" objects="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -6210,7 +6209,28 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="vXCJPiPfq9sOZ4e5mjtWJ21ve7dc7u8UcjEoJ2hDdqZwnTrNL947AnUg1E/49F1PfpQ5MjN/uhsoPc8T+K3vDw==" saltValue="Z2wQx7nSmgQFPTII0GWCdg==" spinCount="100000" sheet="1" objects="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<allowEditUser xmlns="https://web.wps.cn/et/2018/main" xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" hasInvisiblePropRange="0">
+  <rangeList sheetStid="1" master="" otherUserPermission="visible"/>
+  <rangeList sheetStid="2" master="" otherUserPermission="visible"/>
+  <rangeList sheetStid="3" master="" otherUserPermission="visible"/>
+  <rangeList sheetStid="4" master="" otherUserPermission="visible"/>
+  <rangeList sheetStid="5" master="" otherUserPermission="visible"/>
+  <rangeList sheetStid="6" master="" otherUserPermission="visible"/>
+</allowEditUser>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A5607D9-04D2-4DE1-AC0E-A7772F01BC71}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="https://web.wps.cn/et/2018/main"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>